<commit_message>
Add Celestica Q3 2026 entry, update its model and levels
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WkHMtTWpPSAxFWhvppEUAQ
</commit_message>
<xml_diff>
--- a/models/Current_Holdings_DCF.xlsx
+++ b/models/Current_Holdings_DCF.xlsx
@@ -34,9 +34,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1322" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1322" uniqueCount="285">
   <si>
-    <t xml:space="preserve">Current Holdings: scenario values for the 13 stocks</t>
+    <t xml:space="preserve">Current Holdings: scenario values for the 13 stocks (Celestica updated Oct 27, 2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Values link to each company sheet (green). Switch the discount rate on the WACC tab. Funds (JCPI, HYBL, VGK, XBI) are excluded.</t>
@@ -141,7 +141,7 @@
     <t xml:space="preserve">Discount rates use a 5.31% risk-free rate and a 5% equity risk premium, the same as the earlier journal models. At these rates most quality stocks look fully priced; the implied return column shows by how much.</t>
   </si>
   <si>
-    <t xml:space="preserve">Prices: Oct 23, 2026 intraday. Company data: Stock Analysis, company filings and releases (see each sheet). Research for my own records, not investment advice.</t>
+    <t xml:space="preserve">Prices: Oct 23, 2026 intraday, except Celestica (Oct 26 close, model updated for its Q3 results on Oct 27). Company data: Stock Analysis, company filings and releases (see each sheet). Research for my own records, not investment advice.</t>
   </si>
   <si>
     <t xml:space="preserve">Discount rates: calculated (CAPM) versus assumed</t>
@@ -618,16 +618,25 @@
     <t xml:space="preserve">Celestica (CLS): 10-year scenario DCF</t>
   </si>
   <si>
-    <t xml:space="preserve">2026E consensus $20.56B (Stock Analysis); FY27 consensus $35.45B</t>
+    <t xml:space="preserve">Oct 26, 2026 close (before results)</t>
   </si>
   <si>
-    <t xml:space="preserve">Bear: hyperscaler capex cut in 2028</t>
+    <t xml:space="preserve">126.1M shares at Sep 30, 2026, after the August offering of 11.1M shares at $310 (Q3 2026 release)</t>
   </si>
   <si>
-    <t xml:space="preserve">Base: ramp, then mid-single-digit growth</t>
+    <t xml:space="preserve">Q3 2026 release: cash $3,961M less borrowings and leases $819M</t>
   </si>
   <si>
-    <t xml:space="preserve">Bull: share gains in AI networking</t>
+    <t xml:space="preserve">2026 outlook $21.0B (raised from $20.5B, Q3 2026 release). 2027 outlook: $40.0B revenue, 9.0% adjusted operating margin, $21.50 adjusted EPS, $1.5B to $2.0B capex. Margins here are after stock pay, about 0.4 points below adjusted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bear: a large customer pauses, 2027 misses and 2028 falls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base: 2027 lands 8% below the outlook, 2028 grows, 2029 digests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bull: the $40B outlook is met and 2028 is meaningfully higher</t>
   </si>
   <si>
     <t xml:space="preserve">Enterprise Products (EPD): 10-year scenario DCF</t>
@@ -1718,7 +1727,7 @@
       </c>
       <c r="C11" s="4" t="n">
         <f aca="false">CLS!B4</f>
-        <v>264.59</v>
+        <v>246.65</v>
       </c>
       <c r="D11" s="5" t="n">
         <f aca="false">CLS!B10</f>
@@ -1726,23 +1735,23 @@
       </c>
       <c r="E11" s="4" t="n">
         <f aca="false">CLS!B75</f>
-        <v>108.894814907105</v>
+        <v>126.0768383782</v>
       </c>
       <c r="F11" s="4" t="n">
         <f aca="false">CLS!B76</f>
-        <v>201.601478251462</v>
+        <v>198.694451924321</v>
       </c>
       <c r="G11" s="4" t="n">
         <f aca="false">CLS!B77</f>
-        <v>306.393999868867</v>
+        <v>316.918935792392</v>
       </c>
       <c r="H11" s="6" t="n">
         <f aca="false">F11/C11-1</f>
-        <v>-0.238060855468983</v>
+        <v>-0.194427521085259</v>
       </c>
       <c r="I11" s="5" t="n">
         <f aca="false">CLS!B86</f>
-        <v>0.0883097421259398</v>
+        <v>0.0895586861589185</v>
       </c>
       <c r="J11" s="7" t="n">
         <f aca="false">IF(F11&lt;10,ROUND(F11*4,0)/4,IF(F11&lt;100,ROUND(F11,0),ROUND(F11/5,0)*5))</f>
@@ -2050,7 +2059,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2110,7 +2119,7 @@
         <v>0</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2155,7 +2164,7 @@
         <v>58.5</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2288,7 +2297,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="26"/>
@@ -2867,7 +2876,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B37" s="26"/>
       <c r="C37" s="26"/>
@@ -3446,7 +3455,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="12" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B55" s="26"/>
       <c r="C55" s="26"/>
@@ -4271,7 +4280,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4370,13 +4379,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B12" s="22" t="n">
         <v>411.65</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4395,34 +4404,34 @@
         <v>119</v>
       </c>
       <c r="B15" s="24" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="C15" s="24" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="D15" s="24" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="E15" s="24" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="F15" s="24" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="G15" s="24" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="H15" s="24" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="I15" s="24" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="J15" s="24" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="K15" s="24" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="L15" s="9" t="s">
         <v>130</v>
@@ -4509,7 +4518,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="26"/>
@@ -5088,7 +5097,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="B37" s="26"/>
       <c r="C37" s="26"/>
@@ -5667,7 +5676,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="12" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="B55" s="26"/>
       <c r="C55" s="26"/>
@@ -6492,7 +6501,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6552,7 +6561,7 @@
         <v>0</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6597,7 +6606,7 @@
         <v>5.04</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6730,7 +6739,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="26"/>
@@ -7309,7 +7318,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="B37" s="26"/>
       <c r="C37" s="26"/>
@@ -7888,7 +7897,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="12" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B55" s="26"/>
       <c r="C55" s="26"/>
@@ -8711,12 +8720,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8743,18 +8752,18 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B6" s="19" t="n">
         <v>109.96</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B7" s="11" t="n">
         <v>0.6</v>
@@ -8765,7 +8774,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">WACC!B40</f>
@@ -8826,7 +8835,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="B12" s="0" t="n">
         <v>1</v>
@@ -8896,7 +8905,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="B15" s="26"/>
       <c r="C15" s="26"/>
@@ -8912,7 +8921,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B16" s="11" t="n">
         <v>0.17</v>
@@ -8955,7 +8964,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="B17" s="32" t="n">
         <f aca="false">$B$6</f>
@@ -9004,7 +9013,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="B18" s="32" t="n">
         <f aca="false">B16*B17</f>
@@ -9050,7 +9059,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="B19" s="32" t="n">
         <f aca="false">B18*(1-$B$7)</f>
@@ -9096,7 +9105,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="B20" s="32" t="n">
         <f aca="false">(B16-$B$8)*B17</f>
@@ -9191,7 +9200,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="B22" s="32" t="n">
         <f aca="false">B20*B21</f>
@@ -9237,7 +9246,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="B23" s="11" t="n">
         <v>0.035</v>
@@ -9245,7 +9254,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="B24" s="7" t="n">
         <f aca="false">L20/($B$8-B23)/(1+$B$8)^$K$12</f>
@@ -9254,7 +9263,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="B25" s="31" t="n">
         <f aca="false">$B$6+SUM(B22:K22)+B24</f>
@@ -9272,7 +9281,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="B27" s="26"/>
       <c r="C27" s="26"/>
@@ -9288,7 +9297,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B28" s="11" t="n">
         <v>0.2</v>
@@ -9331,7 +9340,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="B29" s="32" t="n">
         <f aca="false">$B$6</f>
@@ -9380,7 +9389,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="B30" s="32" t="n">
         <f aca="false">B28*B29</f>
@@ -9426,7 +9435,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="B31" s="32" t="n">
         <f aca="false">B30*(1-$B$7)</f>
@@ -9472,7 +9481,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="B32" s="32" t="n">
         <f aca="false">(B28-$B$8)*B29</f>
@@ -9567,7 +9576,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="B34" s="32" t="n">
         <f aca="false">B32*B33</f>
@@ -9613,7 +9622,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="B35" s="11" t="n">
         <v>0.04</v>
@@ -9621,7 +9630,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="B36" s="7" t="n">
         <f aca="false">L32/($B$8-B35)/(1+$B$8)^$K$12</f>
@@ -9630,7 +9639,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="B37" s="31" t="n">
         <f aca="false">$B$6+SUM(B34:K34)+B36</f>
@@ -9648,7 +9657,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="12" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="B39" s="26"/>
       <c r="C39" s="26"/>
@@ -9664,7 +9673,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B40" s="11" t="n">
         <v>0.21</v>
@@ -9707,7 +9716,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="B41" s="32" t="n">
         <f aca="false">$B$6</f>
@@ -9756,7 +9765,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="B42" s="32" t="n">
         <f aca="false">B40*B41</f>
@@ -9802,7 +9811,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="B43" s="32" t="n">
         <f aca="false">B42*(1-$B$7)</f>
@@ -9848,7 +9857,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="B44" s="32" t="n">
         <f aca="false">(B40-$B$8)*B41</f>
@@ -9943,7 +9952,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="B46" s="32" t="n">
         <f aca="false">B44*B45</f>
@@ -9989,7 +9998,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="B47" s="11" t="n">
         <v>0.04</v>
@@ -9997,7 +10006,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="B48" s="7" t="n">
         <f aca="false">L44/($B$8-B47)/(1+$B$8)^$K$12</f>
@@ -10006,7 +10015,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="B49" s="31" t="n">
         <f aca="false">$B$6+SUM(B46:K46)+B48</f>
@@ -10094,7 +10103,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="0" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="B57" s="33" t="n">
         <f aca="false">B54/$B$6</f>
@@ -10103,7 +10112,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="B58" s="33" t="n">
         <f aca="false">B4/B6</f>
@@ -10112,7 +10121,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="9" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10249,12 +10258,12 @@
         <v>0.0880383177736682</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
   </sheetData>
@@ -10282,12 +10291,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10314,18 +10323,18 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B6" s="19" t="n">
         <v>29.14</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B7" s="11" t="n">
         <v>0.65</v>
@@ -10336,7 +10345,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">WACC!C40</f>
@@ -10397,7 +10406,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="B12" s="0" t="n">
         <v>1</v>
@@ -10467,7 +10476,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B15" s="26"/>
       <c r="C15" s="26"/>
@@ -10483,7 +10492,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B16" s="11" t="n">
         <v>0.13</v>
@@ -10526,7 +10535,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="B17" s="32" t="n">
         <f aca="false">$B$6</f>
@@ -10575,7 +10584,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="B18" s="32" t="n">
         <f aca="false">B16*B17</f>
@@ -10621,7 +10630,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="B19" s="32" t="n">
         <f aca="false">B18*(1-$B$7)</f>
@@ -10667,7 +10676,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="B20" s="32" t="n">
         <f aca="false">(B16-$B$8)*B17</f>
@@ -10762,7 +10771,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="B22" s="32" t="n">
         <f aca="false">B20*B21</f>
@@ -10808,7 +10817,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="B23" s="11" t="n">
         <v>0.035</v>
@@ -10816,7 +10825,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="B24" s="7" t="n">
         <f aca="false">L20/($B$8-B23)/(1+$B$8)^$K$12</f>
@@ -10825,7 +10834,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="B25" s="31" t="n">
         <f aca="false">$B$6+SUM(B22:K22)+B24</f>
@@ -10843,7 +10852,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="B27" s="26"/>
       <c r="C27" s="26"/>
@@ -10859,7 +10868,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B28" s="11" t="n">
         <v>0.15</v>
@@ -10902,7 +10911,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="B29" s="32" t="n">
         <f aca="false">$B$6</f>
@@ -10951,7 +10960,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="B30" s="32" t="n">
         <f aca="false">B28*B29</f>
@@ -10997,7 +11006,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="0" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="B31" s="32" t="n">
         <f aca="false">B30*(1-$B$7)</f>
@@ -11043,7 +11052,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="B32" s="32" t="n">
         <f aca="false">(B28-$B$8)*B29</f>
@@ -11138,7 +11147,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="B34" s="32" t="n">
         <f aca="false">B32*B33</f>
@@ -11184,7 +11193,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="B35" s="11" t="n">
         <v>0.04</v>
@@ -11192,7 +11201,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="B36" s="7" t="n">
         <f aca="false">L32/($B$8-B35)/(1+$B$8)^$K$12</f>
@@ -11201,7 +11210,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="B37" s="31" t="n">
         <f aca="false">$B$6+SUM(B34:K34)+B36</f>
@@ -11219,7 +11228,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="12" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="B39" s="26"/>
       <c r="C39" s="26"/>
@@ -11235,7 +11244,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="B40" s="11" t="n">
         <v>0.155</v>
@@ -11278,7 +11287,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="B41" s="32" t="n">
         <f aca="false">$B$6</f>
@@ -11327,7 +11336,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="B42" s="32" t="n">
         <f aca="false">B40*B41</f>
@@ -11373,7 +11382,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="B43" s="32" t="n">
         <f aca="false">B42*(1-$B$7)</f>
@@ -11419,7 +11428,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="B44" s="32" t="n">
         <f aca="false">(B40-$B$8)*B41</f>
@@ -11514,7 +11523,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="B46" s="32" t="n">
         <f aca="false">B44*B45</f>
@@ -11560,7 +11569,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="B47" s="11" t="n">
         <v>0.04</v>
@@ -11568,7 +11577,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="B48" s="7" t="n">
         <f aca="false">L44/($B$8-B47)/(1+$B$8)^$K$12</f>
@@ -11577,7 +11586,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="B49" s="31" t="n">
         <f aca="false">$B$6+SUM(B46:K46)+B48</f>
@@ -11665,7 +11674,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="0" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="B57" s="33" t="n">
         <f aca="false">B54/$B$6</f>
@@ -11674,7 +11683,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="B58" s="33" t="n">
         <f aca="false">B4/B6</f>
@@ -11683,7 +11692,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="9" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11820,12 +11829,12 @@
         <v>0.10944482648132</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="2" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
     </row>
   </sheetData>
@@ -11853,12 +11862,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11874,7 +11883,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="B5" s="21" t="n">
         <v>0.44114</v>
@@ -11885,7 +11894,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="B6" s="21" t="n">
         <v>0.09866</v>
@@ -11896,66 +11905,66 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="B7" s="22" t="n">
         <v>5.508</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="B8" s="22" t="n">
         <v>18.1</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="B9" s="17" t="n">
         <v>0.15</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="34" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="B11" s="34" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="C11" s="34" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="D11" s="34" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="E11" s="34" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="F11" s="34" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="G11" s="34" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="H11" s="34" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="B12" s="17" t="n">
         <v>0.4</v>
@@ -11983,7 +11992,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="B13" s="17" t="n">
         <v>0.45</v>
@@ -12011,7 +12020,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="B14" s="17" t="n">
         <v>0.15</v>
@@ -12039,7 +12048,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="B15" s="8" t="n">
         <f aca="false">SUM(B12:B14)</f>
@@ -12052,7 +12061,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="B16" s="0" t="str">
         <f aca="false">IF(ABS(B15-1)&lt;0.0001,"OK","Probabilities must sum to 100%")</f>
@@ -12088,7 +12097,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B20" s="7" t="n">
         <f aca="false">H15</f>
@@ -12114,19 +12123,19 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="B23" s="8" t="n">
         <f aca="false">(B4-G12)/((B13*G13+B14*G14)/(B13+B14)-G12)</f>
         <v>0.664259787597598</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
     </row>
   </sheetData>
@@ -12536,7 +12545,7 @@
       </c>
       <c r="H19" s="5" t="n">
         <f aca="false">CLS!B9</f>
-        <v>0.2</v>
+        <v>0.21</v>
       </c>
       <c r="I19" s="5" t="n">
         <f aca="false">EPD!B9</f>
@@ -12584,7 +12593,7 @@
       </c>
       <c r="H20" s="8" t="n">
         <f aca="false">H18*(1-H19)</f>
-        <v>0.05208</v>
+        <v>0.051429</v>
       </c>
       <c r="I20" s="8" t="n">
         <f aca="false">I18*(1-I19)</f>
@@ -12630,7 +12639,7 @@
       </c>
       <c r="H21" s="15" t="n">
         <f aca="false">CLS!B4*CLS!B6</f>
-        <v>30.4225582</v>
+        <v>31.102565</v>
       </c>
       <c r="I21" s="15" t="n">
         <f aca="false">EPD!B4*EPD!B6</f>
@@ -12671,7 +12680,7 @@
         <v>8.45</v>
       </c>
       <c r="H22" s="16" t="n">
-        <v>0.981</v>
+        <v>0.8188</v>
       </c>
       <c r="I22" s="16" t="n">
         <v>34.21</v>
@@ -12716,7 +12725,7 @@
       </c>
       <c r="H23" s="8" t="n">
         <f aca="false">H21/(H21+H22)</f>
-        <v>0.968761501682316</v>
+        <v>0.974349467825076</v>
       </c>
       <c r="I23" s="8" t="n">
         <f aca="false">I21/(I21+I22)</f>
@@ -12762,7 +12771,7 @@
       </c>
       <c r="H24" s="8" t="n">
         <f aca="false">H22/(H21+H22)</f>
-        <v>0.0312384983176843</v>
+        <v>0.0256505321749242</v>
       </c>
       <c r="I24" s="8" t="n">
         <f aca="false">I22/(I21+I22)</f>
@@ -12808,7 +12817,7 @@
       </c>
       <c r="H25" s="8" t="n">
         <f aca="false">H23*H17+H24*H20</f>
-        <v>0.111891335113866</v>
+        <v>0.112219637647074</v>
       </c>
       <c r="I25" s="8" t="n">
         <f aca="false">I23*I17+I24*I20</f>
@@ -26492,10 +26501,10 @@
         <v>101</v>
       </c>
       <c r="B4" s="19" t="n">
-        <v>264.59</v>
+        <v>246.65</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>102</v>
+        <v>194</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26503,7 +26512,7 @@
         <v>103</v>
       </c>
       <c r="B5" s="20" t="s">
-        <v>104</v>
+        <v>194</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>105</v>
@@ -26514,10 +26523,10 @@
         <v>106</v>
       </c>
       <c r="B6" s="21" t="n">
-        <v>0.11498</v>
+        <v>0.1261</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>61</v>
+        <v>195</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26525,10 +26534,10 @@
         <v>107</v>
       </c>
       <c r="B7" s="22" t="n">
-        <v>-0.44</v>
+        <v>3.1425</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>108</v>
+        <v>196</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26547,7 +26556,7 @@
         <v>72</v>
       </c>
       <c r="B9" s="11" t="n">
-        <v>0.2</v>
+        <v>0.21</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>111</v>
@@ -26581,10 +26590,10 @@
         <v>115</v>
       </c>
       <c r="B12" s="22" t="n">
-        <v>20.56</v>
+        <v>21</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26717,7 +26726,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B19" s="26"/>
       <c r="C19" s="26"/>
@@ -26736,43 +26745,43 @@
         <v>134</v>
       </c>
       <c r="B20" s="22" t="n">
+        <v>33</v>
+      </c>
+      <c r="C20" s="22" t="n">
         <v>28</v>
       </c>
-      <c r="C20" s="22" t="n">
-        <v>25</v>
-      </c>
       <c r="D20" s="22" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E20" s="22" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F20" s="22" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G20" s="27" t="n">
         <f aca="false">F20*(1+$F21+($L21-$F21)*G$17/5)</f>
-        <v>30.8635185185185</v>
+        <v>32.8653448275862</v>
       </c>
       <c r="H20" s="27" t="n">
         <f aca="false">G20*(1+$F21+($L21-$F21)*H$17/5)</f>
-        <v>32.5438656378601</v>
+        <v>34.5539435790725</v>
       </c>
       <c r="I20" s="27" t="n">
         <f aca="false">H20*(1+$F21+($L21-$F21)*I$17/5)</f>
-        <v>33.9962863079942</v>
+        <v>36.0254649694227</v>
       </c>
       <c r="J20" s="27" t="n">
         <f aca="false">I20*(1+$F21+($L21-$F21)*J$17/5)</f>
-        <v>35.1798607201985</v>
+        <v>37.2428772339066</v>
       </c>
       <c r="K20" s="27" t="n">
         <f aca="false">J20*(1+$F21+($L21-$F21)*K$17/5)</f>
-        <v>36.0593572382034</v>
+        <v>38.1739491647543</v>
       </c>
       <c r="L20" s="27" t="n">
         <f aca="false">K20*(1+L21)</f>
-        <v>36.9608411691585</v>
+        <v>39.1282978938731</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26781,39 +26790,39 @@
       </c>
       <c r="B21" s="6" t="n">
         <f aca="false">B20/$B$12-1</f>
-        <v>0.361867704280156</v>
+        <v>0.571428571428571</v>
       </c>
       <c r="C21" s="6" t="n">
         <f aca="false">C20/B20-1</f>
-        <v>-0.107142857142857</v>
+        <v>-0.151515151515152</v>
       </c>
       <c r="D21" s="6" t="n">
         <f aca="false">D20/C20-1</f>
-        <v>0</v>
+        <v>-0.0357142857142857</v>
       </c>
       <c r="E21" s="6" t="n">
         <f aca="false">E20/D20-1</f>
-        <v>0.0800000000000001</v>
+        <v>0.0740740740740742</v>
       </c>
       <c r="F21" s="6" t="n">
         <f aca="false">F20/E20-1</f>
-        <v>0.0740740740740742</v>
+        <v>0.0689655172413792</v>
       </c>
       <c r="G21" s="6" t="n">
         <f aca="false">G20/F20-1</f>
-        <v>0.0642592592592592</v>
+        <v>0.0601724137931035</v>
       </c>
       <c r="H21" s="6" t="n">
         <f aca="false">H20/G20-1</f>
-        <v>0.0544444444444445</v>
+        <v>0.0513793103448275</v>
       </c>
       <c r="I21" s="6" t="n">
         <f aca="false">I20/H20-1</f>
-        <v>0.0446296296296296</v>
+        <v>0.0425862068965517</v>
       </c>
       <c r="J21" s="6" t="n">
         <f aca="false">J20/I20-1</f>
-        <v>0.0348148148148149</v>
+        <v>0.0337931034482759</v>
       </c>
       <c r="K21" s="6" t="n">
         <f aca="false">K20/J20-1</f>
@@ -26834,29 +26843,29 @@
         <v>0.07</v>
       </c>
       <c r="D22" s="29" t="n">
-        <v>0.07</v>
+        <v>0.065</v>
       </c>
       <c r="E22" s="29" t="n">
-        <v>0.07</v>
+        <v>0.065</v>
       </c>
       <c r="F22" s="29" t="n">
-        <v>0.07</v>
+        <v>0.065</v>
       </c>
       <c r="G22" s="6" t="n">
         <f aca="false">$F22+($L22-$F22)*G$17/5</f>
-        <v>0.068</v>
+        <v>0.064</v>
       </c>
       <c r="H22" s="6" t="n">
         <f aca="false">$F22+($L22-$F22)*H$17/5</f>
-        <v>0.066</v>
+        <v>0.063</v>
       </c>
       <c r="I22" s="6" t="n">
         <f aca="false">$F22+($L22-$F22)*I$17/5</f>
-        <v>0.064</v>
+        <v>0.062</v>
       </c>
       <c r="J22" s="6" t="n">
         <f aca="false">$F22+($L22-$F22)*J$17/5</f>
-        <v>0.062</v>
+        <v>0.061</v>
       </c>
       <c r="K22" s="6" t="n">
         <f aca="false">$F22+($L22-$F22)*K$17/5</f>
@@ -26872,47 +26881,47 @@
       </c>
       <c r="B23" s="27" t="n">
         <f aca="false">B20*B22</f>
-        <v>2.24</v>
+        <v>2.64</v>
       </c>
       <c r="C23" s="27" t="n">
         <f aca="false">C20*C22</f>
-        <v>1.75</v>
+        <v>1.96</v>
       </c>
       <c r="D23" s="27" t="n">
         <f aca="false">D20*D22</f>
-        <v>1.75</v>
+        <v>1.755</v>
       </c>
       <c r="E23" s="27" t="n">
         <f aca="false">E20*E22</f>
-        <v>1.89</v>
+        <v>1.885</v>
       </c>
       <c r="F23" s="27" t="n">
         <f aca="false">F20*F22</f>
-        <v>2.03</v>
+        <v>2.015</v>
       </c>
       <c r="G23" s="27" t="n">
         <f aca="false">G20*G22</f>
-        <v>2.09871925925926</v>
+        <v>2.10338206896552</v>
       </c>
       <c r="H23" s="27" t="n">
         <f aca="false">H20*H22</f>
-        <v>2.14789513209877</v>
+        <v>2.17689844548157</v>
       </c>
       <c r="I23" s="27" t="n">
         <f aca="false">I20*I22</f>
-        <v>2.17576232371163</v>
+        <v>2.23357882810421</v>
       </c>
       <c r="J23" s="27" t="n">
         <f aca="false">J20*J22</f>
-        <v>2.1811513646523</v>
+        <v>2.2718155112683</v>
       </c>
       <c r="K23" s="27" t="n">
         <f aca="false">K20*K22</f>
-        <v>2.1635614342922</v>
+        <v>2.29043694988526</v>
       </c>
       <c r="L23" s="27" t="n">
         <f aca="false">L20*L22</f>
-        <v>2.21765047014951</v>
+        <v>2.34769787363239</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26921,47 +26930,47 @@
       </c>
       <c r="B24" s="27" t="n">
         <f aca="false">B23*(1-$B$9)</f>
-        <v>1.792</v>
+        <v>2.0856</v>
       </c>
       <c r="C24" s="27" t="n">
         <f aca="false">C23*(1-$B$9)</f>
-        <v>1.4</v>
+        <v>1.5484</v>
       </c>
       <c r="D24" s="27" t="n">
         <f aca="false">D23*(1-$B$9)</f>
-        <v>1.4</v>
+        <v>1.38645</v>
       </c>
       <c r="E24" s="27" t="n">
         <f aca="false">E23*(1-$B$9)</f>
-        <v>1.512</v>
+        <v>1.48915</v>
       </c>
       <c r="F24" s="27" t="n">
         <f aca="false">F23*(1-$B$9)</f>
-        <v>1.624</v>
+        <v>1.59185</v>
       </c>
       <c r="G24" s="27" t="n">
         <f aca="false">G23*(1-$B$9)</f>
-        <v>1.67897540740741</v>
+        <v>1.66167183448276</v>
       </c>
       <c r="H24" s="27" t="n">
         <f aca="false">H23*(1-$B$9)</f>
-        <v>1.71831610567901</v>
+        <v>1.71974977193044</v>
       </c>
       <c r="I24" s="27" t="n">
         <f aca="false">I23*(1-$B$9)</f>
-        <v>1.7406098589693</v>
+        <v>1.76452727420232</v>
       </c>
       <c r="J24" s="27" t="n">
         <f aca="false">J23*(1-$B$9)</f>
-        <v>1.74492109172184</v>
+        <v>1.79473425390196</v>
       </c>
       <c r="K24" s="27" t="n">
         <f aca="false">K23*(1-$B$9)</f>
-        <v>1.73084914743376</v>
+        <v>1.80944519040935</v>
       </c>
       <c r="L24" s="27" t="n">
         <f aca="false">L23*(1-$B$9)</f>
-        <v>1.77412037611961</v>
+        <v>1.85468132016959</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26969,35 +26978,35 @@
         <v>139</v>
       </c>
       <c r="B25" s="29" t="n">
-        <v>0.015</v>
+        <v>0.035</v>
       </c>
       <c r="C25" s="29" t="n">
-        <v>0.015</v>
+        <v>0.02</v>
       </c>
       <c r="D25" s="29" t="n">
-        <v>0.015</v>
+        <v>0.012</v>
       </c>
       <c r="E25" s="29" t="n">
-        <v>0.015</v>
+        <v>0.012</v>
       </c>
       <c r="F25" s="29" t="n">
-        <v>0.015</v>
+        <v>0.012</v>
       </c>
       <c r="G25" s="6" t="n">
         <f aca="false">$F25+($L25-$F25)*G$17/5</f>
-        <v>0.014</v>
+        <v>0.0116</v>
       </c>
       <c r="H25" s="6" t="n">
         <f aca="false">$F25+($L25-$F25)*H$17/5</f>
-        <v>0.013</v>
+        <v>0.0112</v>
       </c>
       <c r="I25" s="6" t="n">
         <f aca="false">$F25+($L25-$F25)*I$17/5</f>
-        <v>0.012</v>
+        <v>0.0108</v>
       </c>
       <c r="J25" s="6" t="n">
         <f aca="false">$F25+($L25-$F25)*J$17/5</f>
-        <v>0.011</v>
+        <v>0.0104</v>
       </c>
       <c r="K25" s="6" t="n">
         <f aca="false">$F25+($L25-$F25)*K$17/5</f>
@@ -27013,47 +27022,47 @@
       </c>
       <c r="B26" s="27" t="n">
         <f aca="false">B20*B25</f>
-        <v>0.42</v>
+        <v>1.155</v>
       </c>
       <c r="C26" s="27" t="n">
         <f aca="false">C20*C25</f>
-        <v>0.375</v>
+        <v>0.56</v>
       </c>
       <c r="D26" s="27" t="n">
         <f aca="false">D20*D25</f>
-        <v>0.375</v>
+        <v>0.324</v>
       </c>
       <c r="E26" s="27" t="n">
         <f aca="false">E20*E25</f>
-        <v>0.405</v>
+        <v>0.348</v>
       </c>
       <c r="F26" s="27" t="n">
         <f aca="false">F20*F25</f>
-        <v>0.435</v>
+        <v>0.372</v>
       </c>
       <c r="G26" s="27" t="n">
         <f aca="false">G20*G25</f>
-        <v>0.432089259259259</v>
+        <v>0.381238</v>
       </c>
       <c r="H26" s="27" t="n">
         <f aca="false">H20*H25</f>
-        <v>0.423070253292181</v>
+        <v>0.387004168085612</v>
       </c>
       <c r="I26" s="27" t="n">
         <f aca="false">I20*I25</f>
-        <v>0.407955435695931</v>
+        <v>0.389075021669765</v>
       </c>
       <c r="J26" s="27" t="n">
         <f aca="false">J20*J25</f>
-        <v>0.386978467922183</v>
+        <v>0.387325923232629</v>
       </c>
       <c r="K26" s="27" t="n">
         <f aca="false">K20*K25</f>
-        <v>0.360593572382034</v>
+        <v>0.381739491647543</v>
       </c>
       <c r="L26" s="27" t="n">
         <f aca="false">L20*L25</f>
-        <v>0.369608411691585</v>
+        <v>0.391282978938732</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27062,15 +27071,15 @@
       </c>
       <c r="B27" s="27" t="n">
         <f aca="false">$B$11*(B20-$B$12)</f>
-        <v>0.744</v>
+        <v>1.2</v>
       </c>
       <c r="C27" s="27" t="n">
         <f aca="false">$B$11*(C20-B20)</f>
-        <v>-0.3</v>
+        <v>-0.5</v>
       </c>
       <c r="D27" s="27" t="n">
         <f aca="false">$B$11*(D20-C20)</f>
-        <v>0</v>
+        <v>-0.1</v>
       </c>
       <c r="E27" s="27" t="n">
         <f aca="false">$B$11*(E20-D20)</f>
@@ -27082,27 +27091,27 @@
       </c>
       <c r="G27" s="27" t="n">
         <f aca="false">$B$11*(G20-F20)</f>
-        <v>0.186351851851852</v>
+        <v>0.186534482758621</v>
       </c>
       <c r="H27" s="27" t="n">
         <f aca="false">$B$11*(H20-G20)</f>
-        <v>0.168034711934157</v>
+        <v>0.168859875148632</v>
       </c>
       <c r="I27" s="27" t="n">
         <f aca="false">$B$11*(I20-H20)</f>
-        <v>0.145242067013412</v>
+        <v>0.147152139035016</v>
       </c>
       <c r="J27" s="27" t="n">
         <f aca="false">$B$11*(J20-I20)</f>
-        <v>0.118357441220424</v>
+        <v>0.121741226448394</v>
       </c>
       <c r="K27" s="27" t="n">
         <f aca="false">$B$11*(K20-J20)</f>
-        <v>0.0879496518004956</v>
+        <v>0.0931071930847665</v>
       </c>
       <c r="L27" s="27" t="n">
         <f aca="false">$B$11*(L20-K20)</f>
-        <v>0.0901483930955081</v>
+        <v>0.0954348729118856</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27111,47 +27120,47 @@
       </c>
       <c r="B28" s="27" t="n">
         <f aca="false">B24-B26-B27</f>
-        <v>0.628</v>
+        <v>-0.2694</v>
       </c>
       <c r="C28" s="27" t="n">
         <f aca="false">C24-C26-C27</f>
-        <v>1.325</v>
+        <v>1.4884</v>
       </c>
       <c r="D28" s="27" t="n">
         <f aca="false">D24-D26-D27</f>
-        <v>1.025</v>
+        <v>1.16245</v>
       </c>
       <c r="E28" s="27" t="n">
         <f aca="false">E24-E26-E27</f>
-        <v>0.907</v>
+        <v>0.94115</v>
       </c>
       <c r="F28" s="27" t="n">
         <f aca="false">F24-F26-F27</f>
-        <v>0.989</v>
+        <v>1.01985</v>
       </c>
       <c r="G28" s="27" t="n">
         <f aca="false">G24-G26-G27</f>
-        <v>1.0605342962963</v>
+        <v>1.09389935172414</v>
       </c>
       <c r="H28" s="27" t="n">
         <f aca="false">H24-H26-H27</f>
-        <v>1.12721114045267</v>
+        <v>1.1638857286962</v>
       </c>
       <c r="I28" s="27" t="n">
         <f aca="false">I24-I26-I27</f>
-        <v>1.18741235625996</v>
+        <v>1.22830011349754</v>
       </c>
       <c r="J28" s="27" t="n">
         <f aca="false">J24-J26-J27</f>
-        <v>1.23958518257924</v>
+        <v>1.28566710422094</v>
       </c>
       <c r="K28" s="27" t="n">
         <f aca="false">K24-K26-K27</f>
-        <v>1.28230592325123</v>
+        <v>1.33459850567704</v>
       </c>
       <c r="L28" s="27" t="n">
         <f aca="false">L24-L26-L27</f>
-        <v>1.31436357133251</v>
+        <v>1.36796346831897</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27205,43 +27214,43 @@
       </c>
       <c r="B30" s="27" t="n">
         <f aca="false">B28*B29</f>
-        <v>0.597418276658045</v>
+        <v>-0.256281025050441</v>
       </c>
       <c r="C30" s="27" t="n">
         <f aca="false">C28*C29</f>
-        <v>1.14070267828906</v>
+        <v>1.28137499348335</v>
       </c>
       <c r="D30" s="27" t="n">
         <f aca="false">D28*D29</f>
-        <v>0.798579523774463</v>
+        <v>0.905667090157682</v>
       </c>
       <c r="E30" s="27" t="n">
         <f aca="false">E28*E29</f>
-        <v>0.639498181713663</v>
+        <v>0.663576310606189</v>
       </c>
       <c r="F30" s="27" t="n">
         <f aca="false">F28*F29</f>
-        <v>0.631053297594689</v>
+        <v>0.650737821589427</v>
       </c>
       <c r="G30" s="27" t="n">
         <f aca="false">G28*G29</f>
-        <v>0.61239577880673</v>
+        <v>0.631662123304045</v>
       </c>
       <c r="H30" s="27" t="n">
         <f aca="false">H28*H29</f>
-        <v>0.589047700846682</v>
+        <v>0.608212772153259</v>
       </c>
       <c r="I30" s="27" t="n">
         <f aca="false">I28*I29</f>
-        <v>0.561544888934631</v>
+        <v>0.580881314882802</v>
       </c>
       <c r="J30" s="27" t="n">
         <f aca="false">J28*J29</f>
-        <v>0.530514200166688</v>
+        <v>0.550236212131226</v>
       </c>
       <c r="K30" s="27" t="n">
         <f aca="false">K28*K29</f>
-        <v>0.496649505247729</v>
+        <v>0.516902928958084</v>
       </c>
       <c r="L30" s="27"/>
     </row>
@@ -27251,7 +27260,7 @@
       </c>
       <c r="B31" s="27" t="n">
         <f aca="false">L28/($B$10-L21)</f>
-        <v>16.4295446416564</v>
+        <v>17.0995433539871</v>
       </c>
       <c r="C31" s="0" t="str">
         <f aca="false">IF($B$10&gt;L21,"","Discount rate must exceed terminal growth")</f>
@@ -27264,7 +27273,7 @@
       </c>
       <c r="B32" s="27" t="n">
         <f aca="false">B31/(1+$B$10)^$K$16</f>
-        <v>6.36332178598653</v>
+        <v>6.62281877727545</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27273,7 +27282,7 @@
       </c>
       <c r="B33" s="27" t="n">
         <f aca="false">SUM(B30:K30)+B32+$B$7+$B$8</f>
-        <v>12.5207258180189</v>
+        <v>15.8982893194911</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27282,7 +27291,7 @@
       </c>
       <c r="B34" s="31" t="n">
         <f aca="false">B33/$B$6</f>
-        <v>108.894814907105</v>
+        <v>126.0768383782</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27291,12 +27300,12 @@
       </c>
       <c r="B35" s="6" t="n">
         <f aca="false">B34/$B$4-1</f>
-        <v>-0.588439416050853</v>
+        <v>-0.488843144625176</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B37" s="26"/>
       <c r="C37" s="26"/>
@@ -27315,43 +27324,43 @@
         <v>134</v>
       </c>
       <c r="B38" s="22" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="C38" s="22" t="n">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="D38" s="22" t="n">
-        <v>38.5</v>
+        <v>40</v>
       </c>
       <c r="E38" s="22" t="n">
-        <v>40.5</v>
+        <v>42</v>
       </c>
       <c r="F38" s="22" t="n">
-        <v>42.5</v>
+        <v>44</v>
       </c>
       <c r="G38" s="27" t="n">
         <f aca="false">F38*(1+$F39+($L39-$F39)*G$17/5)</f>
-        <v>44.434012345679</v>
+        <v>45.9401904761905</v>
       </c>
       <c r="H38" s="27" t="n">
         <f aca="false">G38*(1+$F39+($L39-$F39)*H$17/5)</f>
-        <v>46.283783822588</v>
+        <v>47.8040496326531</v>
       </c>
       <c r="I38" s="27" t="n">
         <f aca="false">H38*(1+$F39+($L39-$F39)*I$17/5)</f>
-        <v>48.0311395130754</v>
+        <v>49.5750758523771</v>
       </c>
       <c r="J38" s="27" t="n">
         <f aca="false">I38*(1+$F39+($L39-$F39)*J$17/5)</f>
-        <v>49.6582684862097</v>
+        <v>51.2370212523806</v>
       </c>
       <c r="K38" s="27" t="n">
         <f aca="false">J38*(1+$F39+($L39-$F39)*K$17/5)</f>
-        <v>51.1480165407959</v>
+        <v>52.774131889952</v>
       </c>
       <c r="L38" s="27" t="n">
         <f aca="false">K38*(1+L39)</f>
-        <v>52.6824570370198</v>
+        <v>54.3573558466505</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27360,39 +27369,39 @@
       </c>
       <c r="B39" s="6" t="n">
         <f aca="false">B38/$B$12-1</f>
-        <v>0.556420233463035</v>
+        <v>0.761904761904762</v>
       </c>
       <c r="C39" s="6" t="n">
         <f aca="false">C38/B38-1</f>
-        <v>0.15625</v>
+        <v>0.135135135135135</v>
       </c>
       <c r="D39" s="6" t="n">
         <f aca="false">D38/C38-1</f>
-        <v>0.0405405405405406</v>
+        <v>-0.0476190476190477</v>
       </c>
       <c r="E39" s="6" t="n">
         <f aca="false">E38/D38-1</f>
-        <v>0.051948051948052</v>
+        <v>0.05</v>
       </c>
       <c r="F39" s="6" t="n">
         <f aca="false">F38/E38-1</f>
-        <v>0.0493827160493827</v>
+        <v>0.0476190476190477</v>
       </c>
       <c r="G39" s="6" t="n">
         <f aca="false">G38/F38-1</f>
-        <v>0.0455061728395061</v>
+        <v>0.0440952380952382</v>
       </c>
       <c r="H39" s="6" t="n">
         <f aca="false">H38/G38-1</f>
-        <v>0.0416296296296297</v>
+        <v>0.0405714285714287</v>
       </c>
       <c r="I39" s="6" t="n">
         <f aca="false">I38/H38-1</f>
-        <v>0.0377530864197531</v>
+        <v>0.037047619047619</v>
       </c>
       <c r="J39" s="6" t="n">
         <f aca="false">J38/I38-1</f>
-        <v>0.0338765432098764</v>
+        <v>0.0335238095238095</v>
       </c>
       <c r="K39" s="6" t="n">
         <f aca="false">K38/J38-1</f>
@@ -27407,13 +27416,13 @@
         <v>136</v>
       </c>
       <c r="B40" s="29" t="n">
-        <v>0.085</v>
+        <v>0.086</v>
       </c>
       <c r="C40" s="29" t="n">
-        <v>0.085</v>
+        <v>0.086</v>
       </c>
       <c r="D40" s="29" t="n">
-        <v>0.08</v>
+        <v>0.082</v>
       </c>
       <c r="E40" s="29" t="n">
         <v>0.08</v>
@@ -27423,26 +27432,26 @@
       </c>
       <c r="G40" s="6" t="n">
         <f aca="false">$F40+($L40-$F40)*G$17/5</f>
-        <v>0.079</v>
+        <v>0.078</v>
       </c>
       <c r="H40" s="6" t="n">
         <f aca="false">$F40+($L40-$F40)*H$17/5</f>
-        <v>0.078</v>
+        <v>0.076</v>
       </c>
       <c r="I40" s="6" t="n">
         <f aca="false">$F40+($L40-$F40)*I$17/5</f>
-        <v>0.077</v>
+        <v>0.074</v>
       </c>
       <c r="J40" s="6" t="n">
         <f aca="false">$F40+($L40-$F40)*J$17/5</f>
-        <v>0.076</v>
+        <v>0.072</v>
       </c>
       <c r="K40" s="6" t="n">
         <f aca="false">$F40+($L40-$F40)*K$17/5</f>
-        <v>0.075</v>
+        <v>0.07</v>
       </c>
       <c r="L40" s="28" t="n">
-        <v>0.075</v>
+        <v>0.07</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27451,47 +27460,47 @@
       </c>
       <c r="B41" s="27" t="n">
         <f aca="false">B38*B40</f>
-        <v>2.72</v>
+        <v>3.182</v>
       </c>
       <c r="C41" s="27" t="n">
         <f aca="false">C38*C40</f>
-        <v>3.145</v>
+        <v>3.612</v>
       </c>
       <c r="D41" s="27" t="n">
         <f aca="false">D38*D40</f>
-        <v>3.08</v>
+        <v>3.28</v>
       </c>
       <c r="E41" s="27" t="n">
         <f aca="false">E38*E40</f>
-        <v>3.24</v>
+        <v>3.36</v>
       </c>
       <c r="F41" s="27" t="n">
         <f aca="false">F38*F40</f>
-        <v>3.4</v>
+        <v>3.52</v>
       </c>
       <c r="G41" s="27" t="n">
         <f aca="false">G38*G40</f>
-        <v>3.51028697530864</v>
+        <v>3.58333485714286</v>
       </c>
       <c r="H41" s="27" t="n">
         <f aca="false">H38*H40</f>
-        <v>3.61013513816187</v>
+        <v>3.63310777208163</v>
       </c>
       <c r="I41" s="27" t="n">
         <f aca="false">I38*I40</f>
-        <v>3.6983977425068</v>
+        <v>3.6685556130759</v>
       </c>
       <c r="J41" s="27" t="n">
         <f aca="false">J38*J40</f>
-        <v>3.77402840495193</v>
+        <v>3.6890655301714</v>
       </c>
       <c r="K41" s="27" t="n">
         <f aca="false">K38*K40</f>
-        <v>3.8361012405597</v>
+        <v>3.69418923229664</v>
       </c>
       <c r="L41" s="27" t="n">
         <f aca="false">L38*L40</f>
-        <v>3.95118427777649</v>
+        <v>3.80501490926554</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27500,47 +27509,47 @@
       </c>
       <c r="B42" s="27" t="n">
         <f aca="false">B41*(1-$B$9)</f>
-        <v>2.176</v>
+        <v>2.51378</v>
       </c>
       <c r="C42" s="27" t="n">
         <f aca="false">C41*(1-$B$9)</f>
-        <v>2.516</v>
+        <v>2.85348</v>
       </c>
       <c r="D42" s="27" t="n">
         <f aca="false">D41*(1-$B$9)</f>
-        <v>2.464</v>
+        <v>2.5912</v>
       </c>
       <c r="E42" s="27" t="n">
         <f aca="false">E41*(1-$B$9)</f>
-        <v>2.592</v>
+        <v>2.6544</v>
       </c>
       <c r="F42" s="27" t="n">
         <f aca="false">F41*(1-$B$9)</f>
-        <v>2.72</v>
+        <v>2.7808</v>
       </c>
       <c r="G42" s="27" t="n">
         <f aca="false">G41*(1-$B$9)</f>
-        <v>2.80822958024691</v>
+        <v>2.83083453714286</v>
       </c>
       <c r="H42" s="27" t="n">
         <f aca="false">H41*(1-$B$9)</f>
-        <v>2.88810811052949</v>
+        <v>2.87015513994449</v>
       </c>
       <c r="I42" s="27" t="n">
         <f aca="false">I41*(1-$B$9)</f>
-        <v>2.95871819400544</v>
+        <v>2.89815893432996</v>
       </c>
       <c r="J42" s="27" t="n">
         <f aca="false">J41*(1-$B$9)</f>
-        <v>3.01922272396155</v>
+        <v>2.91436176883541</v>
       </c>
       <c r="K42" s="27" t="n">
         <f aca="false">K41*(1-$B$9)</f>
-        <v>3.06888099244776</v>
+        <v>2.91840949351435</v>
       </c>
       <c r="L42" s="27" t="n">
         <f aca="false">L41*(1-$B$9)</f>
-        <v>3.16094742222119</v>
+        <v>3.00596177831978</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27548,10 +27557,10 @@
         <v>139</v>
       </c>
       <c r="B43" s="29" t="n">
-        <v>0.015</v>
+        <v>0.035</v>
       </c>
       <c r="C43" s="29" t="n">
-        <v>0.015</v>
+        <v>0.025</v>
       </c>
       <c r="D43" s="29" t="n">
         <v>0.015</v>
@@ -27592,47 +27601,47 @@
       </c>
       <c r="B44" s="27" t="n">
         <f aca="false">B38*B43</f>
-        <v>0.48</v>
+        <v>1.295</v>
       </c>
       <c r="C44" s="27" t="n">
         <f aca="false">C38*C43</f>
-        <v>0.555</v>
+        <v>1.05</v>
       </c>
       <c r="D44" s="27" t="n">
         <f aca="false">D38*D43</f>
-        <v>0.5775</v>
+        <v>0.6</v>
       </c>
       <c r="E44" s="27" t="n">
         <f aca="false">E38*E43</f>
-        <v>0.6075</v>
+        <v>0.63</v>
       </c>
       <c r="F44" s="27" t="n">
         <f aca="false">F38*F43</f>
-        <v>0.6375</v>
+        <v>0.66</v>
       </c>
       <c r="G44" s="27" t="n">
         <f aca="false">G38*G43</f>
-        <v>0.622076172839506</v>
+        <v>0.643162666666667</v>
       </c>
       <c r="H44" s="27" t="n">
         <f aca="false">H38*H43</f>
-        <v>0.601689189693644</v>
+        <v>0.62145264522449</v>
       </c>
       <c r="I44" s="27" t="n">
         <f aca="false">I38*I43</f>
-        <v>0.576373674156904</v>
+        <v>0.594900910228525</v>
       </c>
       <c r="J44" s="27" t="n">
         <f aca="false">J38*J43</f>
-        <v>0.546240953348306</v>
+        <v>0.563607233776186</v>
       </c>
       <c r="K44" s="27" t="n">
         <f aca="false">K38*K43</f>
-        <v>0.51148016540796</v>
+        <v>0.52774131889952</v>
       </c>
       <c r="L44" s="27" t="n">
         <f aca="false">L38*L43</f>
-        <v>0.526824570370198</v>
+        <v>0.543573558466506</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27641,7 +27650,7 @@
       </c>
       <c r="B45" s="27" t="n">
         <f aca="false">$B$11*(B38-$B$12)</f>
-        <v>1.144</v>
+        <v>1.6</v>
       </c>
       <c r="C45" s="27" t="n">
         <f aca="false">$B$11*(C38-B38)</f>
@@ -27649,7 +27658,7 @@
       </c>
       <c r="D45" s="27" t="n">
         <f aca="false">$B$11*(D38-C38)</f>
-        <v>0.15</v>
+        <v>-0.2</v>
       </c>
       <c r="E45" s="27" t="n">
         <f aca="false">$B$11*(E38-D38)</f>
@@ -27661,27 +27670,27 @@
       </c>
       <c r="G45" s="27" t="n">
         <f aca="false">$B$11*(G38-F38)</f>
-        <v>0.193401234567901</v>
+        <v>0.194019047619048</v>
       </c>
       <c r="H45" s="27" t="n">
         <f aca="false">$B$11*(H38-G38)</f>
-        <v>0.184977147690901</v>
+        <v>0.186385915646259</v>
       </c>
       <c r="I45" s="27" t="n">
         <f aca="false">$B$11*(I38-H38)</f>
-        <v>0.174735569048733</v>
+        <v>0.1771026219724</v>
       </c>
       <c r="J45" s="27" t="n">
         <f aca="false">$B$11*(J38-I38)</f>
-        <v>0.16271289731343</v>
+        <v>0.16619454000035</v>
       </c>
       <c r="K45" s="27" t="n">
         <f aca="false">$B$11*(K38-J38)</f>
-        <v>0.148974805458629</v>
+        <v>0.153711063757142</v>
       </c>
       <c r="L45" s="27" t="n">
         <f aca="false">$B$11*(L38-K38)</f>
-        <v>0.153444049622388</v>
+        <v>0.158322395669856</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27690,47 +27699,47 @@
       </c>
       <c r="B46" s="27" t="n">
         <f aca="false">B42-B44-B45</f>
-        <v>0.552</v>
+        <v>-0.38122</v>
       </c>
       <c r="C46" s="27" t="n">
         <f aca="false">C42-C44-C45</f>
-        <v>1.461</v>
+        <v>1.30348</v>
       </c>
       <c r="D46" s="27" t="n">
         <f aca="false">D42-D44-D45</f>
-        <v>1.7365</v>
+        <v>2.1912</v>
       </c>
       <c r="E46" s="27" t="n">
         <f aca="false">E42-E44-E45</f>
-        <v>1.7845</v>
+        <v>1.8244</v>
       </c>
       <c r="F46" s="27" t="n">
         <f aca="false">F42-F44-F45</f>
-        <v>1.8825</v>
+        <v>1.9208</v>
       </c>
       <c r="G46" s="27" t="n">
         <f aca="false">G42-G44-G45</f>
-        <v>1.99275217283951</v>
+        <v>1.99365282285714</v>
       </c>
       <c r="H46" s="27" t="n">
         <f aca="false">H42-H44-H45</f>
-        <v>2.10144177314495</v>
+        <v>2.06231657907374</v>
       </c>
       <c r="I46" s="27" t="n">
         <f aca="false">I42-I44-I45</f>
-        <v>2.2076089507998</v>
+        <v>2.12615540212904</v>
       </c>
       <c r="J46" s="27" t="n">
         <f aca="false">J42-J44-J45</f>
-        <v>2.31026887329981</v>
+        <v>2.18455999505887</v>
       </c>
       <c r="K46" s="27" t="n">
         <f aca="false">K42-K44-K45</f>
-        <v>2.40842602158117</v>
+        <v>2.23695711085768</v>
       </c>
       <c r="L46" s="27" t="n">
         <f aca="false">L42-L44-L45</f>
-        <v>2.4806788022286</v>
+        <v>2.30406582418341</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27784,43 +27793,43 @@
       </c>
       <c r="B48" s="27" t="n">
         <f aca="false">B46*B47</f>
-        <v>0.525119249546562</v>
+        <v>-0.362655725203153</v>
       </c>
       <c r="C48" s="27" t="n">
         <f aca="false">C46*C47</f>
-        <v>1.25778612300401</v>
+        <v>1.12217594497828</v>
       </c>
       <c r="D48" s="27" t="n">
         <f aca="false">D46*D47</f>
-        <v>1.3529105785701</v>
+        <v>1.7071682463362</v>
       </c>
       <c r="E48" s="27" t="n">
         <f aca="false">E46*E47</f>
-        <v>1.25819680845428</v>
+        <v>1.2863290878924</v>
       </c>
       <c r="F48" s="27" t="n">
         <f aca="false">F46*F47</f>
-        <v>1.20117071053792</v>
+        <v>1.22560887160756</v>
       </c>
       <c r="G48" s="27" t="n">
         <f aca="false">G46*G47</f>
-        <v>1.15069642077271</v>
+        <v>1.15121649284479</v>
       </c>
       <c r="H48" s="27" t="n">
         <f aca="false">H46*H47</f>
-        <v>1.09815224540551</v>
+        <v>1.07770655889147</v>
       </c>
       <c r="I48" s="27" t="n">
         <f aca="false">I46*I47</f>
-        <v>1.0440109676748</v>
+        <v>1.00549037817569</v>
       </c>
       <c r="J48" s="27" t="n">
         <f aca="false">J46*J47</f>
-        <v>0.988742412149882</v>
+        <v>0.934941877962244</v>
       </c>
       <c r="K48" s="27" t="n">
         <f aca="false">K46*K47</f>
-        <v>0.932806727595292</v>
+        <v>0.866395157522945</v>
       </c>
       <c r="L48" s="27"/>
     </row>
@@ -27830,7 +27839,7 @@
       </c>
       <c r="B49" s="27" t="n">
         <f aca="false">L46/($B$10-L39)</f>
-        <v>33.0757173630481</v>
+        <v>30.7208776557789</v>
       </c>
       <c r="C49" s="0" t="str">
         <f aca="false">IF($B$10&gt;L39,"","Discount rate must exceed terminal growth")</f>
@@ -27843,7 +27852,7 @@
       </c>
       <c r="B50" s="27" t="n">
         <f aca="false">B49/(1+$B$10)^$K$16</f>
-        <v>12.810545725642</v>
+        <v>11.8984934966484</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27852,7 +27861,7 @@
       </c>
       <c r="B51" s="27" t="n">
         <f aca="false">SUM(B48:K48)+B50+$B$7+$B$8</f>
-        <v>23.1801379693531</v>
+        <v>25.0553703876569</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27861,7 +27870,7 @@
       </c>
       <c r="B52" s="31" t="n">
         <f aca="false">B51/$B$6</f>
-        <v>201.601478251462</v>
+        <v>198.694451924321</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27870,12 +27879,12 @@
       </c>
       <c r="B53" s="6" t="n">
         <f aca="false">B52/$B$4-1</f>
-        <v>-0.238060855468983</v>
+        <v>-0.194427521085259</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="12" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B55" s="26"/>
       <c r="C55" s="26"/>
@@ -27894,43 +27903,43 @@
         <v>134</v>
       </c>
       <c r="B56" s="22" t="n">
-        <v>35.5</v>
+        <v>40</v>
       </c>
       <c r="C56" s="22" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="D56" s="22" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="E56" s="22" t="n">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="F56" s="22" t="n">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="G56" s="27" t="n">
         <f aca="false">F56*(1+$F57+($L57-$F57)*G$17/5)</f>
-        <v>59.8381538461538</v>
+        <v>65.8546896551724</v>
       </c>
       <c r="H56" s="27" t="n">
         <f aca="false">G56*(1+$F57+($L57-$F57)*H$17/5)</f>
-        <v>63.4376489467456</v>
+        <v>69.5016769512485</v>
       </c>
       <c r="I56" s="27" t="n">
         <f aca="false">H56*(1+$F57+($L57-$F57)*I$17/5)</f>
-        <v>66.7217672345271</v>
+        <v>72.8784998072592</v>
       </c>
       <c r="J56" s="27" t="n">
         <f aca="false">I56*(1+$F57+($L57-$F57)*J$17/5)</f>
-        <v>69.6164654437789</v>
+        <v>75.9243184888591</v>
       </c>
       <c r="K56" s="27" t="n">
         <f aca="false">J56*(1+$F57+($L57-$F57)*K$17/5)</f>
-        <v>72.0530417343111</v>
+        <v>78.5816696359692</v>
       </c>
       <c r="L56" s="27" t="n">
         <f aca="false">K56*(1+L57)</f>
-        <v>74.574898195012</v>
+        <v>81.3320280732281</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -27939,39 +27948,39 @@
       </c>
       <c r="B57" s="6" t="n">
         <f aca="false">B56/$B$12-1</f>
-        <v>0.726653696498055</v>
+        <v>0.904761904761905</v>
       </c>
       <c r="C57" s="6" t="n">
         <f aca="false">C56/B56-1</f>
-        <v>0.211267605633803</v>
+        <v>0.25</v>
       </c>
       <c r="D57" s="6" t="n">
         <f aca="false">D56/C56-1</f>
-        <v>0.116279069767442</v>
+        <v>0.0800000000000001</v>
       </c>
       <c r="E57" s="6" t="n">
         <f aca="false">E56/D56-1</f>
-        <v>0.0833333333333333</v>
+        <v>0.0740740740740742</v>
       </c>
       <c r="F57" s="6" t="n">
         <f aca="false">F56/E56-1</f>
-        <v>0.0769230769230769</v>
+        <v>0.0689655172413792</v>
       </c>
       <c r="G57" s="6" t="n">
         <f aca="false">G56/F56-1</f>
-        <v>0.0685384615384614</v>
+        <v>0.0621724137931035</v>
       </c>
       <c r="H57" s="6" t="n">
         <f aca="false">H56/G56-1</f>
-        <v>0.0601538461538462</v>
+        <v>0.0553793103448275</v>
       </c>
       <c r="I57" s="6" t="n">
         <f aca="false">I56/H56-1</f>
-        <v>0.0517692307692308</v>
+        <v>0.0485862068965517</v>
       </c>
       <c r="J57" s="6" t="n">
         <f aca="false">J56/I56-1</f>
-        <v>0.0433846153846154</v>
+        <v>0.0417931034482759</v>
       </c>
       <c r="K57" s="6" t="n">
         <f aca="false">K56/J56-1</f>
@@ -27986,7 +27995,7 @@
         <v>136</v>
       </c>
       <c r="B58" s="29" t="n">
-        <v>0.09</v>
+        <v>0.088</v>
       </c>
       <c r="C58" s="29" t="n">
         <v>0.09</v>
@@ -27998,23 +28007,23 @@
         <v>0.09</v>
       </c>
       <c r="F58" s="29" t="n">
-        <v>0.085</v>
+        <v>0.088</v>
       </c>
       <c r="G58" s="6" t="n">
         <f aca="false">$F58+($L58-$F58)*G$17/5</f>
-        <v>0.084</v>
+        <v>0.0864</v>
       </c>
       <c r="H58" s="6" t="n">
         <f aca="false">$F58+($L58-$F58)*H$17/5</f>
-        <v>0.083</v>
+        <v>0.0848</v>
       </c>
       <c r="I58" s="6" t="n">
         <f aca="false">$F58+($L58-$F58)*I$17/5</f>
-        <v>0.082</v>
+        <v>0.0832</v>
       </c>
       <c r="J58" s="6" t="n">
         <f aca="false">$F58+($L58-$F58)*J$17/5</f>
-        <v>0.081</v>
+        <v>0.0816</v>
       </c>
       <c r="K58" s="6" t="n">
         <f aca="false">$F58+($L58-$F58)*K$17/5</f>
@@ -28030,47 +28039,47 @@
       </c>
       <c r="B59" s="27" t="n">
         <f aca="false">B56*B58</f>
-        <v>3.195</v>
+        <v>3.52</v>
       </c>
       <c r="C59" s="27" t="n">
         <f aca="false">C56*C58</f>
-        <v>3.87</v>
+        <v>4.5</v>
       </c>
       <c r="D59" s="27" t="n">
         <f aca="false">D56*D58</f>
-        <v>4.32</v>
+        <v>4.86</v>
       </c>
       <c r="E59" s="27" t="n">
         <f aca="false">E56*E58</f>
-        <v>4.68</v>
+        <v>5.22</v>
       </c>
       <c r="F59" s="27" t="n">
         <f aca="false">F56*F58</f>
-        <v>4.76</v>
+        <v>5.456</v>
       </c>
       <c r="G59" s="27" t="n">
         <f aca="false">G56*G58</f>
-        <v>5.02640492307692</v>
+        <v>5.6898451862069</v>
       </c>
       <c r="H59" s="27" t="n">
         <f aca="false">H56*H58</f>
-        <v>5.26532486257988</v>
+        <v>5.89374220546587</v>
       </c>
       <c r="I59" s="27" t="n">
         <f aca="false">I56*I58</f>
-        <v>5.47118491323122</v>
+        <v>6.06349118396396</v>
       </c>
       <c r="J59" s="27" t="n">
         <f aca="false">J56*J58</f>
-        <v>5.63893370094609</v>
+        <v>6.1954243886909</v>
       </c>
       <c r="K59" s="27" t="n">
         <f aca="false">K56*K58</f>
-        <v>5.76424333874489</v>
+        <v>6.28653357087753</v>
       </c>
       <c r="L59" s="27" t="n">
         <f aca="false">L56*L58</f>
-        <v>5.96599185560096</v>
+        <v>6.50656224585825</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28079,47 +28088,47 @@
       </c>
       <c r="B60" s="27" t="n">
         <f aca="false">B59*(1-$B$9)</f>
-        <v>2.556</v>
+        <v>2.7808</v>
       </c>
       <c r="C60" s="27" t="n">
         <f aca="false">C59*(1-$B$9)</f>
-        <v>3.096</v>
+        <v>3.555</v>
       </c>
       <c r="D60" s="27" t="n">
         <f aca="false">D59*(1-$B$9)</f>
-        <v>3.456</v>
+        <v>3.8394</v>
       </c>
       <c r="E60" s="27" t="n">
         <f aca="false">E59*(1-$B$9)</f>
-        <v>3.744</v>
+        <v>4.1238</v>
       </c>
       <c r="F60" s="27" t="n">
         <f aca="false">F59*(1-$B$9)</f>
-        <v>3.808</v>
+        <v>4.31024</v>
       </c>
       <c r="G60" s="27" t="n">
         <f aca="false">G59*(1-$B$9)</f>
-        <v>4.02112393846154</v>
+        <v>4.49497769710345</v>
       </c>
       <c r="H60" s="27" t="n">
         <f aca="false">H59*(1-$B$9)</f>
-        <v>4.21225989006391</v>
+        <v>4.65605634231804</v>
       </c>
       <c r="I60" s="27" t="n">
         <f aca="false">I59*(1-$B$9)</f>
-        <v>4.37694793058498</v>
+        <v>4.79015803533153</v>
       </c>
       <c r="J60" s="27" t="n">
         <f aca="false">J59*(1-$B$9)</f>
-        <v>4.51114696075687</v>
+        <v>4.89438526706581</v>
       </c>
       <c r="K60" s="27" t="n">
         <f aca="false">K59*(1-$B$9)</f>
-        <v>4.61139467099591</v>
+        <v>4.96636152099325</v>
       </c>
       <c r="L60" s="27" t="n">
         <f aca="false">L59*(1-$B$9)</f>
-        <v>4.77279348448077</v>
+        <v>5.14018417422802</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28127,13 +28136,13 @@
         <v>139</v>
       </c>
       <c r="B61" s="29" t="n">
-        <v>0.015</v>
+        <v>0.04</v>
       </c>
       <c r="C61" s="29" t="n">
-        <v>0.015</v>
+        <v>0.03</v>
       </c>
       <c r="D61" s="29" t="n">
-        <v>0.015</v>
+        <v>0.02</v>
       </c>
       <c r="E61" s="29" t="n">
         <v>0.015</v>
@@ -28171,47 +28180,47 @@
       </c>
       <c r="B62" s="27" t="n">
         <f aca="false">B56*B61</f>
-        <v>0.5325</v>
+        <v>1.6</v>
       </c>
       <c r="C62" s="27" t="n">
         <f aca="false">C56*C61</f>
-        <v>0.645</v>
+        <v>1.5</v>
       </c>
       <c r="D62" s="27" t="n">
         <f aca="false">D56*D61</f>
-        <v>0.72</v>
+        <v>1.08</v>
       </c>
       <c r="E62" s="27" t="n">
         <f aca="false">E56*E61</f>
-        <v>0.78</v>
+        <v>0.87</v>
       </c>
       <c r="F62" s="27" t="n">
         <f aca="false">F56*F61</f>
-        <v>0.84</v>
+        <v>0.93</v>
       </c>
       <c r="G62" s="27" t="n">
         <f aca="false">G56*G61</f>
-        <v>0.837734153846154</v>
+        <v>0.921965655172414</v>
       </c>
       <c r="H62" s="27" t="n">
         <f aca="false">H56*H61</f>
-        <v>0.824689436307692</v>
+        <v>0.90352180036623</v>
       </c>
       <c r="I62" s="27" t="n">
         <f aca="false">I56*I61</f>
-        <v>0.800661206814325</v>
+        <v>0.87454199768711</v>
       </c>
       <c r="J62" s="27" t="n">
         <f aca="false">J56*J61</f>
-        <v>0.765781119881568</v>
+        <v>0.83516750337745</v>
       </c>
       <c r="K62" s="27" t="n">
         <f aca="false">K56*K61</f>
-        <v>0.720530417343111</v>
+        <v>0.785816696359692</v>
       </c>
       <c r="L62" s="27" t="n">
         <f aca="false">L56*L61</f>
-        <v>0.74574898195012</v>
+        <v>0.813320280732281</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28220,15 +28229,15 @@
       </c>
       <c r="B63" s="27" t="n">
         <f aca="false">$B$11*(B56-$B$12)</f>
-        <v>1.494</v>
+        <v>1.9</v>
       </c>
       <c r="C63" s="27" t="n">
         <f aca="false">$B$11*(C56-B56)</f>
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="D63" s="27" t="n">
         <f aca="false">$B$11*(D56-C56)</f>
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="E63" s="27" t="n">
         <f aca="false">$B$11*(E56-D56)</f>
@@ -28240,27 +28249,27 @@
       </c>
       <c r="G63" s="27" t="n">
         <f aca="false">$B$11*(G56-F56)</f>
-        <v>0.383815384615384</v>
+        <v>0.385468965517241</v>
       </c>
       <c r="H63" s="27" t="n">
         <f aca="false">$B$11*(H56-G56)</f>
-        <v>0.359949510059172</v>
+        <v>0.364698729607609</v>
       </c>
       <c r="I63" s="27" t="n">
         <f aca="false">$B$11*(I56-H56)</f>
-        <v>0.328411828778152</v>
+        <v>0.337682285601066</v>
       </c>
       <c r="J63" s="27" t="n">
         <f aca="false">$B$11*(J56-I56)</f>
-        <v>0.289469820925179</v>
+        <v>0.304581868159994</v>
       </c>
       <c r="K63" s="27" t="n">
         <f aca="false">$B$11*(K56-J56)</f>
-        <v>0.243657629053226</v>
+        <v>0.265735114711006</v>
       </c>
       <c r="L63" s="27" t="n">
         <f aca="false">$B$11*(L56-K56)</f>
-        <v>0.252185646070089</v>
+        <v>0.275035843725891</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28269,47 +28278,47 @@
       </c>
       <c r="B64" s="27" t="n">
         <f aca="false">B60-B62-B63</f>
-        <v>0.5295</v>
+        <v>-0.719200000000001</v>
       </c>
       <c r="C64" s="27" t="n">
         <f aca="false">C60-C62-C63</f>
-        <v>1.701</v>
+        <v>1.055</v>
       </c>
       <c r="D64" s="27" t="n">
         <f aca="false">D60-D62-D63</f>
-        <v>2.236</v>
+        <v>2.3594</v>
       </c>
       <c r="E64" s="27" t="n">
         <f aca="false">E60-E62-E63</f>
-        <v>2.564</v>
+        <v>2.8538</v>
       </c>
       <c r="F64" s="27" t="n">
         <f aca="false">F60-F62-F63</f>
-        <v>2.568</v>
+        <v>2.98024</v>
       </c>
       <c r="G64" s="27" t="n">
         <f aca="false">G60-G62-G63</f>
-        <v>2.7995744</v>
+        <v>3.18754307641379</v>
       </c>
       <c r="H64" s="27" t="n">
         <f aca="false">H60-H62-H63</f>
-        <v>3.02762094369704</v>
+        <v>3.3878358123442</v>
       </c>
       <c r="I64" s="27" t="n">
         <f aca="false">I60-I62-I63</f>
-        <v>3.2478748949925</v>
+        <v>3.57793375204335</v>
       </c>
       <c r="J64" s="27" t="n">
         <f aca="false">J60-J62-J63</f>
-        <v>3.45589601995012</v>
+        <v>3.75463589552837</v>
       </c>
       <c r="K64" s="27" t="n">
         <f aca="false">K60-K62-K63</f>
-        <v>3.64720662459958</v>
+        <v>3.91480970992255</v>
       </c>
       <c r="L64" s="27" t="n">
         <f aca="false">L60-L62-L63</f>
-        <v>3.77485885646056</v>
+        <v>4.05182804976984</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28363,43 +28372,43 @@
       </c>
       <c r="B66" s="27" t="n">
         <f aca="false">B64*B65</f>
-        <v>0.503714932309609</v>
+        <v>-0.684177109191825</v>
       </c>
       <c r="C66" s="27" t="n">
         <f aca="false">C64*C65</f>
-        <v>1.46440396661863</v>
+        <v>0.908257604222609</v>
       </c>
       <c r="D66" s="27" t="n">
         <f aca="false">D64*D65</f>
-        <v>1.74207201478995</v>
+        <v>1.83821319843265</v>
       </c>
       <c r="E66" s="27" t="n">
         <f aca="false">E64*E65</f>
-        <v>1.80779860850478</v>
+        <v>2.0121277960027</v>
       </c>
       <c r="F66" s="27" t="n">
         <f aca="false">F64*F65</f>
-        <v>1.63856912863818</v>
+        <v>1.90160796726349</v>
       </c>
       <c r="G66" s="27" t="n">
         <f aca="false">G64*G65</f>
-        <v>1.61658849789464</v>
+        <v>1.84061744309215</v>
       </c>
       <c r="H66" s="27" t="n">
         <f aca="false">H64*H65</f>
-        <v>1.58214649582314</v>
+        <v>1.77038429136354</v>
       </c>
       <c r="I66" s="27" t="n">
         <f aca="false">I64*I65</f>
-        <v>1.53596813909426</v>
+        <v>1.69205786078816</v>
       </c>
       <c r="J66" s="27" t="n">
         <f aca="false">J64*J65</f>
-        <v>1.4790447148362</v>
+        <v>1.60689857141467</v>
       </c>
       <c r="K66" s="27" t="n">
         <f aca="false">K64*K65</f>
-        <v>1.41259845470489</v>
+        <v>1.51624372181201</v>
       </c>
       <c r="L66" s="27"/>
     </row>
@@ -28409,7 +28418,7 @@
       </c>
       <c r="B67" s="27" t="n">
         <f aca="false">L64/($B$10-L57)</f>
-        <v>53.9265550922937</v>
+        <v>57.8832578538549</v>
       </c>
       <c r="C67" s="0" t="str">
         <f aca="false">IF($B$10&gt;L57,"","Discount rate must exceed terminal growth")</f>
@@ -28422,7 +28431,7 @@
       </c>
       <c r="B68" s="27" t="n">
         <f aca="false">B67/(1+$B$10)^$K$16</f>
-        <v>20.886277151708</v>
+        <v>22.4187464582205</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28431,7 +28440,7 @@
       </c>
       <c r="B69" s="27" t="n">
         <f aca="false">SUM(B66:K66)+B68+$B$7+$B$8</f>
-        <v>35.2291821049223</v>
+        <v>39.9634778034207</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28440,7 +28449,7 @@
       </c>
       <c r="B70" s="31" t="n">
         <f aca="false">B69/$B$6</f>
-        <v>306.393999868867</v>
+        <v>316.918935792392</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28449,7 +28458,7 @@
       </c>
       <c r="B71" s="6" t="n">
         <f aca="false">B70/$B$4-1</f>
-        <v>0.157995388596949</v>
+        <v>0.284893313571426</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28476,11 +28485,11 @@
       </c>
       <c r="B75" s="7" t="n">
         <f aca="false">B34</f>
-        <v>108.894814907105</v>
+        <v>126.0768383782</v>
       </c>
       <c r="C75" s="6" t="n">
         <f aca="false">B75/$B$4-1</f>
-        <v>-0.588439416050853</v>
+        <v>-0.488843144625176</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28489,11 +28498,11 @@
       </c>
       <c r="B76" s="7" t="n">
         <f aca="false">B52</f>
-        <v>201.601478251462</v>
+        <v>198.694451924321</v>
       </c>
       <c r="C76" s="6" t="n">
         <f aca="false">B76/$B$4-1</f>
-        <v>-0.238060855468983</v>
+        <v>-0.194427521085259</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28502,11 +28511,11 @@
       </c>
       <c r="B77" s="7" t="n">
         <f aca="false">B70</f>
-        <v>306.393999868867</v>
+        <v>316.918935792392</v>
       </c>
       <c r="C77" s="6" t="n">
         <f aca="false">B77/$B$4-1</f>
-        <v>0.157995388596949</v>
+        <v>0.284893313571426</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28515,11 +28524,11 @@
       </c>
       <c r="B78" s="7" t="n">
         <f aca="false">INDEX(B34:B70,1+($B$13-1)*18)</f>
-        <v>201.601478251462</v>
+        <v>198.694451924321</v>
       </c>
       <c r="C78" s="6" t="n">
         <f aca="false">B78/$B$4-1</f>
-        <v>-0.238060855468983</v>
+        <v>-0.194427521085259</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28528,7 +28537,7 @@
       </c>
       <c r="B79" s="8" t="n">
         <f aca="false">B50/(SUM(B48:K48)+B50)</f>
-        <v>0.54235693890796</v>
+        <v>0.54299109546829</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28577,43 +28586,43 @@
       </c>
       <c r="B83" s="7" t="n">
         <f aca="false">IF(B82&gt;$L39,(SUMPRODUCT($B46:$K46/(1+B82)^$B$16:$K$16)+$L46/(B82-$L39)/(1+B82)^$K$16+$B$7+$B$8)/$B$6,"n/a")</f>
-        <v>797.201554806562</v>
+        <v>704.39451039781</v>
       </c>
       <c r="C83" s="7" t="n">
         <f aca="false">IF(C82&gt;$L39,(SUMPRODUCT($B46:$K46/(1+C82)^$B$16:$K$16)+$L46/(C82-$L39)/(1+C82)^$K$16+$B$7+$B$8)/$B$6,"n/a")</f>
-        <v>526.018371099413</v>
+        <v>474.46434067676</v>
       </c>
       <c r="D83" s="7" t="n">
         <f aca="false">IF(D82&gt;$L39,(SUMPRODUCT($B46:$K46/(1+D82)^$B$16:$K$16)+$L46/(D82-$L39)/(1+D82)^$K$16+$B$7+$B$8)/$B$6,"n/a")</f>
-        <v>390.591284758548</v>
+        <v>359.520959051058</v>
       </c>
       <c r="E83" s="7" t="n">
         <f aca="false">IF(E82&gt;$L39,(SUMPRODUCT($B46:$K46/(1+E82)^$B$16:$K$16)+$L46/(E82-$L39)/(1+E82)^$K$16+$B$7+$B$8)/$B$6,"n/a")</f>
-        <v>309.457574986465</v>
+        <v>290.572659028855</v>
       </c>
       <c r="F83" s="7" t="n">
         <f aca="false">IF(F82&gt;$L39,(SUMPRODUCT($B46:$K46/(1+F82)^$B$16:$K$16)+$L46/(F82-$L39)/(1+F82)^$K$16+$B$7+$B$8)/$B$6,"n/a")</f>
-        <v>255.463631123386</v>
+        <v>244.622139994527</v>
       </c>
       <c r="G83" s="7" t="n">
         <f aca="false">IF(G82&gt;$L39,(SUMPRODUCT($B46:$K46/(1+G82)^$B$16:$K$16)+$L46/(G82-$L39)/(1+G82)^$K$16+$B$7+$B$8)/$B$6,"n/a")</f>
-        <v>216.972679860817</v>
+        <v>211.813367100302</v>
       </c>
       <c r="H83" s="7" t="n">
         <f aca="false">IF(H82&gt;$L39,(SUMPRODUCT($B46:$K46/(1+H82)^$B$16:$K$16)+$L46/(H82-$L39)/(1+H82)^$K$16+$B$7+$B$8)/$B$6,"n/a")</f>
-        <v>188.16672175981</v>
+        <v>187.218285496945</v>
       </c>
       <c r="I83" s="7" t="n">
         <f aca="false">IF(I82&gt;$L39,(SUMPRODUCT($B46:$K46/(1+I82)^$B$16:$K$16)+$L46/(I82-$L39)/(1+I82)^$K$16+$B$7+$B$8)/$B$6,"n/a")</f>
-        <v>165.813847135179</v>
+        <v>168.099057834869</v>
       </c>
       <c r="J83" s="7" t="n">
         <f aca="false">IF(J82&gt;$L39,(SUMPRODUCT($B46:$K46/(1+J82)^$B$16:$K$16)+$L46/(J82-$L39)/(1+J82)^$K$16+$B$7+$B$8)/$B$6,"n/a")</f>
-        <v>147.975165371079</v>
+        <v>152.812958811803</v>
       </c>
       <c r="K83" s="7" t="n">
         <f aca="false">IF(K82&gt;$L39,(SUMPRODUCT($B46:$K46/(1+K82)^$B$16:$K$16)+$L46/(K82-$L39)/(1+K82)^$K$16+$B$7+$B$8)/$B$6,"n/a")</f>
-        <v>133.41704790957</v>
+        <v>140.314599607172</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28622,43 +28631,43 @@
       </c>
       <c r="B84" s="6" t="n">
         <f aca="false">IFERROR(B83/$B$4-1,"n/a")</f>
-        <v>2.01296932917556</v>
+        <v>1.85584638312512</v>
       </c>
       <c r="C84" s="6" t="n">
         <f aca="false">IFERROR(C83/$B$4-1,"n/a")</f>
-        <v>0.988050837519984</v>
+        <v>0.923634059098967</v>
       </c>
       <c r="D84" s="6" t="n">
         <f aca="false">IFERROR(D83/$B$4-1,"n/a")</f>
-        <v>0.476213329145273</v>
+        <v>0.457615889118419</v>
       </c>
       <c r="E84" s="6" t="n">
         <f aca="false">IFERROR(E83/$B$4-1,"n/a")</f>
-        <v>0.169573963439529</v>
+        <v>0.178076866121449</v>
       </c>
       <c r="F84" s="6" t="n">
         <f aca="false">IFERROR(F83/$B$4-1,"n/a")</f>
-        <v>-0.0344924935810631</v>
+        <v>-0.00822160959040197</v>
       </c>
       <c r="G84" s="6" t="n">
         <f aca="false">IFERROR(G83/$B$4-1,"n/a")</f>
-        <v>-0.179966439166948</v>
+        <v>-0.141239136021482</v>
       </c>
       <c r="H84" s="6" t="n">
         <f aca="false">IFERROR(H83/$B$4-1,"n/a")</f>
-        <v>-0.288836608489323</v>
+        <v>-0.240955663908595</v>
       </c>
       <c r="I84" s="6" t="n">
         <f aca="false">IFERROR(I83/$B$4-1,"n/a")</f>
-        <v>-0.373317785497641</v>
+        <v>-0.318471283864304</v>
       </c>
       <c r="J84" s="6" t="n">
         <f aca="false">IFERROR(J83/$B$4-1,"n/a")</f>
-        <v>-0.440737876068336</v>
+        <v>-0.380446143069925</v>
       </c>
       <c r="K84" s="6" t="n">
         <f aca="false">IFERROR(K83/$B$4-1,"n/a")</f>
-        <v>-0.495759295855589</v>
+        <v>-0.431118590686511</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28667,7 +28676,7 @@
       </c>
       <c r="B86" s="18" t="n">
         <f aca="false">IFERROR(IF(MATCH($B$4,$B$83:$K$83,-1)=10,"above 14%",INDEX($B$82:$K$82,MATCH($B$4,$B$83:$K$83,-1))+(INDEX($B$83:$K$83,MATCH($B$4,$B$83:$K$83,-1))-$B$4)/(INDEX($B$83:$K$83,MATCH($B$4,$B$83:$K$83,-1))-INDEX($B$83:$K$83,MATCH($B$4,$B$83:$K$83,-1)+1))*(INDEX($B$82:$K$82,MATCH($B$4,$B$83:$K$83,-1)+1)-INDEX($B$82:$K$82,MATCH($B$4,$B$83:$K$83,-1)))),"below 5%")</f>
-        <v>0.0883097421259398</v>
+        <v>0.0895586861589185</v>
       </c>
       <c r="C86" s="2" t="s">
         <v>162</v>

</xml_diff>